<commit_message>
updating portfolio_copilot and small changes in other files
</commit_message>
<xml_diff>
--- a/data/Classical_Result.xlsx
+++ b/data/Classical_Result.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,12 +442,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VNQ</t>
+          <t>TLT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>REIT</t>
+          <t>Bond</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -460,12 +460,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TLT</t>
+          <t>VNQ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bond</t>
+          <t>REIT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -478,16 +478,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>REET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>REIT</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -496,12 +496,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DBC</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Commodity</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -514,18 +514,108 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REET</t>
+          <t>SLV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>REIT</t>
+          <t>Commodity</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>0.01</v>
       </c>
       <c r="D6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>REIT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DBC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Commodity</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -577,22 +667,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1454812297068934</v>
+        <v>0.1176468692590703</v>
       </c>
       <c r="B2" t="n">
-        <v>3.821</v>
+        <v>3.8301</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006548621482187168</v>
+        <v>0.008589379235336403</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09381464980422281</v>
+        <v>0.08894504424189535</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0009669999999999999</v>
+        <v>0.0009979999999999998</v>
       </c>
       <c r="F2" t="n">
-        <v>83.71782347794492</v>
+        <v>97.25364227549498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding technical document in docs folder
</commit_message>
<xml_diff>
--- a/data/Classical_Result.xlsx
+++ b/data/Classical_Result.xlsx
@@ -478,12 +478,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REET</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>REIT</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -496,12 +496,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>SLV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Commodity</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -514,7 +514,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SLV</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -568,12 +568,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>REET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>REIT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -667,22 +667,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.1176468692590703</v>
+        <v>0.1512900966413651</v>
       </c>
       <c r="B2" t="n">
-        <v>3.8301</v>
+        <v>3.7393</v>
       </c>
       <c r="C2" t="n">
-        <v>0.008589379235336403</v>
+        <v>0.006385634225163031</v>
       </c>
       <c r="D2" t="n">
-        <v>0.08894504424189535</v>
+        <v>0.09811726844786775</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0009979999999999998</v>
+        <v>0.0009790000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>97.25364227549498</v>
+        <v>82.36170054033371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>